<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-08 La miette de la couverture
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-08.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-08.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, maman</t>
+          <t>Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut garder une miette pour l'ours, dans le seau bleu. Le vent soulève la couverture. Avant de rentrer, elle reprend seau, manteau et ours.</t>
+          <t>La chaise gratte. Sur la couverture à carreaux, un éclat de carreau luit. Une miette s'arrête dessus. Nina veut le pique-nique du square, maintenant. Elle ramasse tout d'un coup : seau, ours, manteau s'emmêlent, l'éclat disparaît. Papa s'accroupit. Seau, manteau, ours. Merci vécu. Au square, elle part avec l'ours seul. Elle refuse de foncer, revient vers l'éclat. Sur la chaise, l'éclat de carreau reste pâle et sablé.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur la chaise, une couverture à carreaux attend. Elle a encore des miettes de pain. Maman la secoue au-dessus de l'évier. Les miettes tombent. On emporte la couverture, Nina ? Oui. Pour s'asseoir. Pour le pique-nique. Maman plie la couverture. Le tissu est doux, un peu rêche. On va au square ? Oui. Avec l'ours. Ils marchent. Le sac sent le pain. En ce moment, Nina est au square. La couverture est déjà posée dans l'herbe. Je m'assois dessus. Nina a un seau bleu. Elle a un manteau jaune. Elle a son doudou ours. Le vent fraîchit. J'ai mangé le pain, maman. Oui. Il reste une miette. Nina la montre. C'est pour l'ours. Elle la pose dans le seau bleu. Tu as encore faim ? Non. Je joue. Elle verse le sable dans le seau. Ça fait chh. La miette reste au fond. Le vent soulève un coin de la couverture. Je le tiens. Merci, maman. Le vent fraîchit. On rentre. La couverture aussi ? Oui. On reprend ses affaires, avant de partir. Nina s'arrête. Elle cherche le seau près du bac. Elle le prend. Le seau bleu. La miette est dedans. Bien. Le manteau est sur la couverture. L'ours est dans l'herbe. L'herbe chatouille.</t>
+          <t>La chaise de la cuisine gratte le carrelage. Au dossier, la couverture à carreaux pend. Un éclat de carreau luit, pâle, au bord. Il brille, papa. C'est un carreau plus clair. Le pain tiède sent le four. L'air sent la croûte, près de l'évier. Une miette roule vers toi, Nina. La miette s'arrête pile sur l'éclat. C'est le pain de l'ours ! L'ours brun attend près du seau bleu. On emporte la couverture, Nina ? Oui, le square, maintenant ! Avec le seau, et ton manteau. Le manteau jaune attend près de la porte. Le zip du manteau fait un petit clic. En ce moment, Nina ramasse tout d'un coup. Ours, seau et manteau s'emmêlent. Le seau tape le carrelage, toc. Ça tombe ! La couverture glisse et cache l'éclat. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sur la chaise, une couverture à carreaux attend. Elle a encore des miettes de pain. Maman la secoue au-dessus de l'évier. Les miettes tombent. On emporte la couverture, Nina ? Oui. Pour s'asseoir. Pour le pique-nique. Maman plie la couverture. Le tissu est doux, un peu rêche. On va au square ? Oui. Avec l'ours. Ils marchent. Le sac sent le pain. En ce moment, Nina est au square. La couverture est déjà posée dans l'herbe. Je m'assois dessus. Nina a un seau bleu. Elle a un manteau jaune. Elle a son doudou ours. Le vent fraîchit. J'ai mangé le pain, maman. Oui. Il reste une miette. Nina la montre. C'est pour l'ours. Elle la pose dans le seau bleu. Tu as encore faim ? Non. Je joue. Elle verse le sable dans le seau. Ça fait chh. La miette reste au fond. Le vent soulève un coin de la couverture. Je le tiens. Merci, maman. Le vent fraîchit. On rentre. La couverture aussi ? Oui. On reprend ses affaires, avant de partir. Nina s'arrête. Elle cherche le seau près du bac. Elle le prend. Le seau bleu. La miette est dedans. Bien. Le manteau est sur la couverture. L'ours est dans l'herbe. L'herbe chatouille.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La chaise de la cuisine gratte le carrelage. Au dossier, la couverture à carreaux pend. Un &lt;emphasis level="moderate"&gt;éclat de carreau&lt;/emphasis&gt; luit, pâle, au bord. Il brille, papa. C'est un carreau plus clair. Le pain tiède sent le four. L'air sent la croûte, près de l'évier. Une miette roule vers toi, Nina. La miette s'arrête pile sur l'éclat. C'est le pain de l'ours ! L'ours brun attend près du seau bleu. On emporte la couverture, Nina ? Oui, le square, maintenant ! Avec le seau, et ton manteau. Le manteau jaune attend près de la porte. Le zip du manteau fait un petit clic. En ce moment, Nina ramasse tout d'un coup. Ours, seau et manteau s'emmêlent. Le seau tape le carrelage, toc. Ça tombe ! La couverture glisse et cache l'éclat. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ariane a pique-niqué au square. Maman est sur la couverture. Ariane a un seau bleu. Elle a un manteau jaune. Elle a son doudou ours. Le vent fraîchit. Maman dit : on rentre. Maman dit : on va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires, avant de partir. Parce qu'on rentre, Ariane s'arrête. Elle cherche le seau près du bac. Elle le prend. Elle cherche le manteau sur la couverture. Elle le prend. Elle cherche le doudou dans l'herbe. L'herbe chatouille. Elle le prend. Maintenant Ariane a tout. Maman dit : merci. Avant de partir, on reprend ses affaires. Ariane marche vers la maison. Le doudou est dans son bras. [pause]</t>
+          <t>La chaise de la cuisine gratte le carrelage. Au dossier, la couverture à carreaux pend. Un &lt;emphasis&gt;éclat de carreau&lt;/emphasis&gt; luit, pâle, au bord. Il brille, papa. C'est un carreau plus clair. Le pain tiède sent le four. L'air sent la croûte, près de l'évier. Une miette roule vers toi, Nina. La miette s'arrête pile sur l'éclat. C'est le pain de l'ours ! L'ours brun attend près du seau bleu. On emporte la couverture, Nina ? Oui, le square, maintenant ! Avec le seau, et ton manteau. Le manteau jaune attend près de la porte. Le zip du manteau fait un petit clic. En ce moment, Nina ramasse tout d'un coup. Ours, seau et manteau s'emmêlent. Le seau tape le carrelage, toc. Ça tombe ! La couverture glisse et cache l'éclat. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>éclat de carreau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,65 +1326,41 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_pique_nique_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Sur la chaise, une couverture à carreaux attend.
-narrateur|Elle a encore des miettes de pain.
-narrateur|Maman la secoue au-dessus de l'évier.
-narrateur|Les miettes tombent.
+          <t>narrateur|La chaise de la cuisine gratte le carrelage.
+narrateur|Au dossier, la couverture à carreaux pend.
+narrateur|Un éclat de carreau luit, pâle, au bord.
+enfant-f|Il brille, papa.
+papa|C'est un carreau plus clair.
+narrateur|Le pain tiède sent le four.
+narrateur|L'air sent la croûte, près de l'évier.
+papa|Une miette roule vers toi, Nina.
+narrateur|La miette s'arrête pile sur l'éclat.
+enfant-f|C'est le pain de l'ours !
+narrateur|L'ours brun attend près du seau bleu.
 maman|On emporte la couverture, Nina ?
-enfant-f|Oui.
-enfant-f|Pour s'asseoir.
-maman|Pour le pique-nique.
-narrateur|Maman plie la couverture.
-narrateur|Le tissu est doux, un peu rêche.
-maman|On va au square ?
-enfant-f|Oui.
-enfant-f|Avec l'ours.
-narrateur|Ils marchent.
-narrateur|Le sac sent le pain.
-narrateur|En ce moment, Nina est au square.
-narrateur|La couverture est déjà posée dans l'herbe.
-maman|Je m'assois dessus.
-narrateur|Nina a un seau bleu.
-narrateur|Elle a un manteau jaune.
-narrateur|Elle a son doudou ours.
-narrateur|Le vent fraîchit.
-enfant-f|J'ai mangé le pain, maman.
-maman|Oui.
-maman|Il reste une miette.
-narrateur|Nina la montre.
-enfant-f|C'est pour l'ours.
-narrateur|Elle la pose dans le seau bleu.
-maman|Tu as encore faim ?
-enfant-f|Non.
-enfant-f|Je joue.
-narrateur|Elle verse le sable dans le seau.
-narrateur|Ça fait chh.
-narrateur|La miette reste au fond.
-narrateur|Le vent soulève un coin de la couverture.
-maman|Je le tiens.
-enfant-f|Merci, maman.
-maman|Le vent fraîchit.
-maman|On rentre.
-enfant-f|La couverture aussi ?
-maman|Oui.
-maman|On reprend ses affaires, avant de partir.
-narrateur|Nina s'arrête.
-narrateur|Elle cherche le seau près du bac.
-narrateur|Elle le prend.
-enfant-f|Le seau bleu.
-enfant-f|La miette est dedans.
-maman|Bien.
-narrateur|Le manteau est sur la couverture.
-narrateur|L'ours est dans l'herbe.
-narrateur|L'herbe chatouille.</t>
+enfant-f|Oui, le square, maintenant !
+maman|Avec le seau, et ton manteau.
+narrateur|Le manteau jaune attend près de la porte.
+narrateur|Le zip du manteau fait un petit clic.
+narrateur|En ce moment, Nina ramasse tout d'un coup.
+narrateur|Ours, seau et manteau s'emmêlent.
+narrateur|Le seau tape le carrelage, toc.
+enfant-f|Ça tombe !
+narrateur|La couverture glisse et cache l'éclat.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>chaise,pain,seau</t>
         </is>
       </c>
     </row>
@@ -1411,17 +1387,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Nina ?</t>
+          <t>Nina veut partir au square. Avant de partir, que fait Nina ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Nina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina veut &lt;emphasis level="moderate"&gt;partir&lt;/emphasis&gt; au square. Avant de partir, que fait Nina ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir, que fait Ariane ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina veut &lt;emphasis&gt;partir&lt;/emphasis&gt; au square. Avant de partir, que fait Nina ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1484,7 +1460,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1495,7 +1471,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1510,38 +1486,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>partir</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1556,22 +1532,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_reprend_ses_affaires_avant_de_partir; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, que fait Nina ?</t>
+          <t>narrateur|Nina veut partir au square.
+narrateur|Avant de partir, que fait Nina ?</t>
         </is>
       </c>
     </row>
@@ -1598,17 +1575,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina cherche le manteau. Elle le prend sur la couverture. Il est jaune. Et l'ours ? Elle cherche le doudou dans l'herbe. L'herbe chatouille. Elle le prend. L'ours est là. Tu as repris tes affaires. Avant de partir. Oui. La miette vient aussi. Maintenant Nina a tout. Maman plie la couverture. Nina marche vers la maison. Le doudou est dans son bras. Tu tiens le seau ? Oui, maman.</t>
+          <t>Papa s'accroupit à la même hauteur. Le seau d'abord, Nina. Nina ramasse le seau bleu. Le plastique est un peu rêche. Le manteau, après le seau. Elle prend le manteau jaune. Et mon ours ? Regarde sous la couverture ? Nina soulève un coin du tissu. L'éclat de carreau reparaît, pâle. La miette est collée au carreau clair. Ma miette est là. L'ours est blotti contre l'éclat. Il était caché. Elle glisse l'ours sous son bras. Merci, Nina. On y va ? Tu as le seau ? Oui, maman. Maman plie la couverture, coin par coin. Nina pose la main sur le tissu. Sous les doigts, l'éclat de carreau reste froid. Le square n'est pas loin. Le sac sent le pain, sur le chemin. L'air dehors sent l'herbe coupée.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina cherche le manteau. Elle le prend sur la couverture. Il est jaune. Et l'ours ? Elle cherche le doudou dans l'herbe. L'herbe chatouille. Elle le prend. L'ours est là. Tu as repris tes affaires. Avant de partir. Oui. La miette vient aussi. Maintenant Nina a tout. Maman plie la couverture. Nina marche vers la maison. Le doudou est dans son bras. Tu tiens le seau ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa s'accroupit à la même hauteur. Le seau d'abord, Nina. Nina ramasse le seau bleu. Le plastique est un peu rêche. Le manteau, après le seau. Elle prend le manteau jaune. Et mon ours ? Regarde sous la couverture ? Nina soulève un coin du tissu. L'&lt;emphasis level="moderate"&gt;éclat de carreau&lt;/emphasis&gt; reparaît, pâle. La miette est collée au carreau clair. Ma miette est là. L'ours est blotti contre l'éclat. Il était caché. Elle glisse l'ours sous son bras. Merci, Nina. On y va ? Tu as le seau ? Oui, maman. Maman plie la couverture, coin par coin. Nina pose la main sur le tissu. Sous les doigts, l'éclat de carreau reste froid. Le square n'est pas loin. Le sac sent le pain, sur le chemin. L'air dehors sent l'herbe coupée.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ariane a cherché. Elle a repris ses affaires. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir. [pause]</t>
+          <t>Papa s'accroupit à la même hauteur. Le seau d'abord, Nina. Nina ramasse le seau bleu. Le plastique est un peu rêche. Le manteau, après le seau. Elle prend le manteau jaune. Et mon ours ? Regarde sous la couverture ? Nina soulève un coin du tissu. L'&lt;emphasis&gt;éclat de carreau&lt;/emphasis&gt; reparaît, pâle. La miette est collée au carreau clair. Ma miette est là. L'ours est blotti contre l'éclat. Il était caché. Elle glisse l'ours sous son bras. Merci, Nina. On y va ? Tu as le seau ? Oui, maman. Maman plie la couverture, coin par coin. Nina pose la main sur le tissu. Sous les doigts, l'éclat de carreau reste froid. Le square n'est pas loin. Le sac sent le pain, sur le chemin. L'air dehors sent l'herbe coupée. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1666,7 +1643,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1689,7 +1666,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>éclat de carreau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1703,16 +1680,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1737,29 +1714,41 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=seau_puis_manteau_puis_ours; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina cherche le manteau.
-narrateur|Elle le prend sur la couverture.
-enfant-f|Il est jaune.
-maman|Et l'ours ?
-narrateur|Elle cherche le doudou dans l'herbe.
-narrateur|L'herbe chatouille.
-narrateur|Elle le prend.
-enfant-f|L'ours est là.
-maman|Tu as repris tes affaires.
-enfant-f|Avant de partir.
-maman|Oui.
-maman|La miette vient aussi.
-narrateur|Maintenant Nina a tout.
-narrateur|Maman plie la couverture.
-narrateur|Nina marche vers la maison.
-narrateur|Le doudou est dans son bras.
-maman|Tu tiens le seau ?
-enfant-f|Oui, maman.</t>
+          <t>narrateur|Papa s'accroupit à la même hauteur.
+papa|Le seau d'abord, Nina.
+narrateur|Nina ramasse le seau bleu.
+narrateur|Le plastique est un peu rêche.
+maman|Le manteau, après le seau.
+narrateur|Elle prend le manteau jaune.
+enfant-f|Et mon ours ?
+papa|Regarde sous la couverture ?
+narrateur|Nina soulève un coin du tissu.
+narrateur|L'éclat de carreau reparaît, pâle.
+narrateur|La miette est collée au carreau clair.
+enfant-f|Ma miette est là.
+narrateur|L'ours est blotti contre l'éclat.
+enfant-f|Il était caché.
+narrateur|Elle glisse l'ours sous son bras.
+papa|Merci, Nina.
+enfant-f|On y va ?
+maman|Tu as le seau ?
+enfant-f|Oui, maman.
+narrateur|Maman plie la couverture, coin par coin.
+narrateur|Nina pose la main sur le tissu.
+narrateur|Sous les doigts, l'éclat de carreau reste froid.
+papa|Le square n'est pas loin.
+narrateur|Le sac sent le pain, sur le chemin.
+narrateur|L'air dehors sent l'herbe coupée.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>zip,seau</t>
         </is>
       </c>
     </row>
@@ -1786,17 +1775,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina marche près de maman. Le seau tape sa jambe. Ils arrivent à la cuisine. Maman pose la couverture sur la chaise. Tu poses le seau près de la porte ? Nina pose le seau. Elle pose le manteau. L'ours reste contre elle. La miette ? On la met dans une soucoupe. Nina cherche au fond du seau. La miette est un peu sableuse. Je la prends. Maman la pose dans la soucoupe. Nina assied l'ours devant. C'est son pain. Bravo. Tu as repris tes affaires. Une autre miette reste sur la chaise. Je la prends. Plus de miettes. Plus de miettes.</t>
+          <t>Au square, l'herbe chatouille les chevilles. On pose la couverture ici ? Oui, pour s'asseoir. Nina étale le tissu dans l'herbe. L'éclat de carreau luit vers le ciel. La miette, pour l'ours. Elle pose la miette sur l'éclat. Il a son pain, lui. Nina verse du sable dans le seau. Ça fait chh, autour de la miette. Mon château, maintenant ! Le vent fraîchit, soulève un coin. Je le tiens ! On rentre, le vent pique. J'y vais avec l'ours ! Elle part, l'ours contre la joue. Le seau reste près du bac. Le manteau reste sur le tissu. Ma miette ! Nina s'arrête net. Elle refuse de foncer. Attends, je regarde. Sur la couverture, l'éclat de carreau pâlit. La miette est là, minuscule. Tu la vois, sur le carreau ? Oui. Elle revient, prend le seau. La sangle tape sa jambe. Elle reprend le manteau jaune. Et la couverture ? Oui, je la tiens.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nina marche près de maman. Le seau tape sa jambe. Ils arrivent à la cuisine. Maman pose la couverture sur la chaise. Tu poses le seau près de la porte ? Nina pose le seau. Elle pose le manteau. L'ours reste contre elle. La miette ? On la met dans une soucoupe. Nina cherche au fond du seau. La miette est un peu sableuse. Je la prends. Maman la pose dans la soucoupe. Nina assied l'ours devant. C'est son pain. Bravo. Tu as repris tes affaires. Une autre miette reste sur la chaise. Je la prends. Plus de miettes. Plus de miettes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au square, l'herbe chatouille les chevilles. On pose la couverture ici ? Oui, pour s'asseoir. Nina étale le tissu dans l'herbe. L'&lt;emphasis level="moderate"&gt;éclat de carreau&lt;/emphasis&gt; luit vers le ciel. La miette, pour l'ours. Elle pose la miette sur l'éclat. Il a son pain, lui. Nina verse du sable dans le seau. Ça fait chh, autour de la miette. Mon château, maintenant ! Le vent fraîchit, soulève un coin. Je le tiens ! On rentre, le vent pique. J'y vais avec l'ours ! Elle part, l'ours contre la joue. Le seau reste près du bac. Le manteau reste sur le tissu. Ma miette ! Nina s'arrête net. Elle refuse de foncer. Attends, je regarde. Sur la couverture, l'éclat de carreau pâlit. La miette est là, minuscule. Tu la vois, sur le carreau ? Oui. Elle revient, prend le seau. La sangle tape sa jambe. Elle reprend le manteau jaune. Et la couverture ? Oui, je la tiens.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ariane marche près de maman. Le seau tape sa jambe. [pause]</t>
+          <t>Au square, l'herbe chatouille les chevilles. On pose la couverture ici ? Oui, pour s'asseoir. Nina étale le tissu dans l'herbe. L'&lt;emphasis&gt;éclat de carreau&lt;/emphasis&gt; luit vers le ciel. La miette, pour l'ours. Elle pose la miette sur l'éclat. Il a son pain, lui. Nina verse du sable dans le seau. Ça fait chh, autour de la miette. Mon château, maintenant ! Le vent fraîchit, soulève un coin. Je le tiens ! On rentre, le vent pique. J'y vais avec l'ours ! Elle part, l'ours contre la joue. Le seau reste près du bac. Le manteau reste sur le tissu. Ma miette ! Nina s'arrête net. Elle refuse de foncer. Attends, je regarde. Sur la couverture, l'éclat de carreau pâlit. La miette est là, minuscule. Tu la vois, sur le carreau ? Oui. Elle revient, prend le seau. La sangle tape sa jambe. Elle reprend le manteau jaune. Et la couverture ? Oui, je la tiens. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1843,7 +1832,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1851,10 +1840,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1875,28 +1864,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de carreau</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1905,10 +1898,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1919,31 +1912,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sans_la_miette; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nina marche près de maman.
-narrateur|Le seau tape sa jambe.
-narrateur|Ils arrivent à la cuisine.
-narrateur|Maman pose la couverture sur la chaise.
-maman|Tu poses le seau près de la porte ?
-narrateur|Nina pose le seau.
-narrateur|Elle pose le manteau.
-narrateur|L'ours reste contre elle.
-enfant-f|La miette ?
-maman|On la met dans une soucoupe.
-narrateur|Nina cherche au fond du seau.
-narrateur|La miette est un peu sableuse.
-maman|Je la prends.
-narrateur|Maman la pose dans la soucoupe.
-narrateur|Nina assied l'ours devant.
-enfant-f|C'est son pain.
-maman|Bravo.
-maman|Tu as repris tes affaires.
-narrateur|Une autre miette reste sur la chaise.
-maman|Je la prends.
-enfant-f|Plus de miettes.
-maman|Plus de miettes.</t>
+          <t>narrateur|Au square, l'herbe chatouille les chevilles.
+maman|On pose la couverture ici ?
+enfant-f|Oui, pour s'asseoir.
+narrateur|Nina étale le tissu dans l'herbe.
+narrateur|L'éclat de carreau luit vers le ciel.
+enfant-f|La miette, pour l'ours.
+narrateur|Elle pose la miette sur l'éclat.
+papa|Il a son pain, lui.
+narrateur|Nina verse du sable dans le seau.
+narrateur|Ça fait chh, autour de la miette.
+enfant-f|Mon château, maintenant !
+narrateur|Le vent fraîchit, soulève un coin.
+enfant-f|Je le tiens !
+maman|On rentre, le vent pique.
+enfant-f|J'y vais avec l'ours !
+narrateur|Elle part, l'ours contre la joue.
+narrateur|Le seau reste près du bac.
+narrateur|Le manteau reste sur le tissu.
+enfant-f|Ma miette !
+narrateur|Nina s'arrête net.
+narrateur|Elle refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Sur la couverture, l'éclat de carreau pâlit.
+narrateur|La miette est là, minuscule.
+papa|Tu la vois, sur le carreau ?
+enfant-f|Oui.
+narrateur|Elle revient, prend le seau.
+narrateur|La sangle tape sa jambe.
+narrateur|Elle reprend le manteau jaune.
+maman|Et la couverture ?
+enfant-f|Oui, je la tiens.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>herbe,vent,seau</t>
         </is>
       </c>
     </row>
@@ -1970,17 +1981,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'ours a sa miette. Et toi, tu as repris tes affaires. La couverture à carreaux repose.</t>
+          <t>La cuisine sent le pain, au retour. Maman pose la couverture sur la chaise. L'éclat de carreau luit, comme au départ. La miette ? Regarde l'éclat, Nina. Nina se penche vers le tissu. La miette est sableuse, collée à l'éclat. Elle a tenu. Nina assied l'ours devant le tissu. C'est son pain. Tu le vois, le petit éclat ? Oui, maman. Le seau bleu repose près de la porte. Le manteau jaune retrouve le crochet. Sur la chaise, l'éclat de carreau reste pâle et sablé.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>L'ours a sa miette. Et toi, tu as repris tes affaires. La couverture à carreaux repose.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La cuisine sent le pain, au retour. Maman pose la couverture sur la chaise. L'&lt;emphasis level="moderate"&gt;éclat de carreau&lt;/emphasis&gt; luit, comme au départ. La miette ? Regarde l'éclat, Nina. Nina se penche vers le tissu. La miette est sableuse, collée à l'éclat. Elle a tenu. Nina assied l'ours devant le tissu. C'est son pain. Tu le vois, le petit éclat ? Oui, maman. Le seau bleu repose près de la porte. Le manteau jaune retrouve le crochet. Sur la chaise, l'éclat de carreau reste pâle et sablé.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La cuisine sent le pain, au retour. Maman pose la couverture sur la chaise. L'&lt;emphasis&gt;éclat de carreau&lt;/emphasis&gt; luit, comme au départ. La miette ? Regarde l'éclat, Nina. Nina se penche vers le tissu. La miette est sableuse, collée à l'éclat. Elle a tenu. Nina assied l'ours devant le tissu. C'est son pain. Tu le vois, le petit éclat ? Oui, maman. Le seau bleu repose près de la porte. Le manteau jaune retrouve le crochet. Sur la chaise, l'éclat de carreau reste pâle et sablé.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2027,7 +2038,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2035,10 +2046,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2047,12 +2058,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2061,17 +2072,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de carreau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2080,11 +2095,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2093,26 +2108,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=la_miette_repose_sur_l_eclat_du_debut; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|L'ours a sa miette.
-maman|Et toi, tu as repris tes affaires.
-narrateur|La couverture à carreaux repose.</t>
+          <t>narrateur|La cuisine sent le pain, au retour.
+narrateur|Maman pose la couverture sur la chaise.
+narrateur|L'éclat de carreau luit, comme au départ.
+enfant-f|La miette ?
+papa|Regarde l'éclat, Nina.
+narrateur|Nina se penche vers le tissu.
+narrateur|La miette est sableuse, collée à l'éclat.
+enfant-f|Elle a tenu.
+narrateur|Nina assied l'ours devant le tissu.
+enfant-f|C'est son pain.
+maman|Tu le vois, le petit éclat ?
+enfant-f|Oui, maman.
+narrateur|Le seau bleu repose près de la porte.
+narrateur|Le manteau jaune retrouve le crochet.
+narrateur|Sur la chaise, l'éclat de carreau reste pâle et sablé.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>chaise,pain</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2225,6 +2261,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>